<commit_message>
new UI new look
</commit_message>
<xml_diff>
--- a/data/templates/po_template.xlsx
+++ b/data/templates/po_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cc\PO-generator\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A16CDB89-9B6F-4648-B171-35AAAABACB19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF8FFA8-B4D5-4390-9D77-226ACC737E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-5205" windowWidth="29040" windowHeight="15720" tabRatio="523" xr2:uid="{3D730B16-2E6A-4D13-B9C1-6FB9A054ACE9}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="130">
   <si>
     <t>TO:</t>
   </si>
@@ -69,12 +69,42 @@
     <t>UNIT</t>
   </si>
   <si>
+    <t>a)</t>
+  </si>
+  <si>
+    <t>Supplier shall consign the goods to :-</t>
+  </si>
+  <si>
     <t>b)</t>
   </si>
   <si>
     <t>A copy of the Suppliers proposed Packing List and Shipping</t>
   </si>
   <si>
+    <t>The Packing List and Shipping Invoice shall clearly state :-</t>
+  </si>
+  <si>
+    <t>Dubai-L.L.C. P.O.Box 4613 Dubai - U.A.E</t>
+  </si>
+  <si>
+    <t>Manufactures Data Requirements</t>
+  </si>
+  <si>
+    <t>Quality Requirements</t>
+  </si>
+  <si>
+    <t>Spare Parts And Interchangeability List (Blank )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Innovative Technologies (Syntech) Ltd. General Purchase Terms And </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice shall be faxed to Innovative Technologies (Syntech) Ltd.  prior to </t>
+  </si>
+  <si>
+    <t>shipment of goods from the point of origin for approval.</t>
+  </si>
+  <si>
     <t>PLEASE SIGN AND RETURN AN ACCEPTANCE COPY OF THIS P.O. WITHIN THREE DAYS OF RECEIPT.</t>
   </si>
   <si>
@@ -87,18 +117,161 @@
     <t>Date:</t>
   </si>
   <si>
+    <t xml:space="preserve">All test, inspection and certification documents shall be handled according to note-2. </t>
+  </si>
+  <si>
+    <t>Supplier is requested to fully complete the commissioning spare parts list attached to this purchase order.</t>
+  </si>
+  <si>
+    <t>expediting of equipment covered by this purchase order throughout duration of the order.</t>
+  </si>
+  <si>
     <t>Supplier Ref:</t>
   </si>
   <si>
+    <t>3c</t>
+  </si>
+  <si>
+    <t>Supplier to advise the single point of contact (Name, Address, Phone, Fax &amp; e-mail ID) at the factory/works</t>
+  </si>
+  <si>
+    <t>Attachments to this purchase order</t>
+  </si>
+  <si>
+    <t>8a</t>
+  </si>
+  <si>
+    <t>8b</t>
+  </si>
+  <si>
+    <t>8c</t>
+  </si>
+  <si>
+    <t>8d</t>
+  </si>
+  <si>
+    <t>For items covered by this purchase order the following shall apply unless otherwise stated:-</t>
+  </si>
+  <si>
+    <t>9a</t>
+  </si>
+  <si>
+    <t>9b</t>
+  </si>
+  <si>
+    <t>9c</t>
+  </si>
+  <si>
+    <t>3d</t>
+  </si>
+  <si>
+    <t>9d</t>
+  </si>
+  <si>
+    <t>9e</t>
+  </si>
+  <si>
+    <t>Material Request</t>
+  </si>
+  <si>
+    <t>8e</t>
+  </si>
+  <si>
     <t>DEFINITIONS</t>
   </si>
   <si>
+    <t>Purchaser and/or their nominated representative, client reserves the right to carry out testing/inspection,</t>
+  </si>
+  <si>
     <t>TERMS OF DELIVERY</t>
   </si>
   <si>
+    <t>Copy of following documents shall be emailed/faxed to Purchaser Prior to shipment of goods from the</t>
+  </si>
+  <si>
+    <t>point of origin for purchasers approval.</t>
+  </si>
+  <si>
     <t>TERMS OF PAYMENT</t>
   </si>
   <si>
+    <t>Manufacturers Data Requirements</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Packing List, Shipping Invoice. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>No material shall be depatched without the approval of above documents</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Supplier is requested to fully complete the 2 years operating spare parts and interchangeability list </t>
+  </si>
+  <si>
+    <t>attached to this purchase order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commissioning spare parts shall be packed separately and clearly marked with part numbers and shall </t>
+  </si>
+  <si>
+    <t>be shipped along with the consignment.</t>
+  </si>
+  <si>
+    <t>Applicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The equipment covered by this Purchase Order is part of an EPCC Contract awarded to Purchaser as </t>
+  </si>
+  <si>
+    <t xml:space="preserve">such timely delivery of documents and equipment is critical to Purchaser's overall schedule. </t>
+  </si>
+  <si>
+    <t>be fully packed, suitable for the export shipment.</t>
+  </si>
+  <si>
+    <t>Failure by the Supplier to fully comply with the above requirement may result in importation duties being</t>
+  </si>
+  <si>
+    <t xml:space="preserve">incurred by Purchaser, which may not subsequently be recoverable. In such event Purchaser reserves the </t>
+  </si>
+  <si>
+    <t>"The equipment/materials listed is to be exported out of Malaysia.</t>
+  </si>
+  <si>
+    <t>right to backcharge the Supplier with all associated costs.</t>
+  </si>
+  <si>
+    <t>Material release certificate issued by Suppliers QC department or Purchaser's representative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Applicable</t>
+  </si>
+  <si>
+    <t>Not  Applicable</t>
+  </si>
+  <si>
+    <r>
+      <t>Supplier shall consign the goods to:-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">          </t>
+    </r>
+  </si>
+  <si>
     <t>Name :</t>
   </si>
   <si>
@@ -111,6 +284,9 @@
     <t>Project :</t>
   </si>
   <si>
+    <t xml:space="preserve">Unless otherwise instructed, all shipments are to be dispatched for airfreight / shipment. All equipment shall </t>
+  </si>
+  <si>
     <t xml:space="preserve">Supplier -  </t>
   </si>
   <si>
@@ -123,10 +299,25 @@
     <t xml:space="preserve">TOTAL PRICE   </t>
   </si>
   <si>
+    <t>DIRECTOR - GENERAL MANAGER</t>
+  </si>
+  <si>
     <t>Notes:</t>
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>All correspondence associated with this purchase order shall be addressed to:</t>
+  </si>
+  <si>
+    <t>Purchase Order No.:</t>
+  </si>
+  <si>
+    <t>All Manufacturers data associated with this purchase order shall be addressed to :-</t>
+  </si>
+  <si>
+    <t>Inspections, Testing and Certification requirements shall be providied</t>
   </si>
   <si>
     <t>Total amount  of order in words</t>
@@ -173,12 +364,45 @@
     <t xml:space="preserve">Email        </t>
   </si>
   <si>
+    <t>C-3A-03, Pusat Perdagangan Phileo Damansara 1,</t>
+  </si>
+  <si>
+    <t>Tel No.  : +603 79315799</t>
+  </si>
+  <si>
+    <t>Fax No. : n/a</t>
+  </si>
+  <si>
+    <t>As per Quadex Automation Sdn Bhd General Purchase Terms and Conditions</t>
+  </si>
+  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
+    <t>The Procurement Manager: QUADEX AUTOMATION SDN BHD, C-3A-03, Pusat Perdagangan Phileo Damansara 1, Jalan 16/11, 46350, Petaling Jaya</t>
+  </si>
+  <si>
+    <t>The Document Controller:QUADEX AUTOMATION SDN BHD, C-3A-03, Pusat Perdagangan Phileo Damansara 1, Jalan 16/11, 46350, Petaling Jaya</t>
+  </si>
+  <si>
+    <t>Quadex Automation Sdn Bhd General Purchase Terms And Conditions</t>
+  </si>
+  <si>
+    <t>QUADEX AUTOMATION SDN BHD, C-3A-03, Pusat Perdagangan Phileo Damansara 1, Jalan 16/11, 46350, Petaling Jaya</t>
+  </si>
+  <si>
     <t>Page 1 of 2</t>
   </si>
   <si>
+    <t>Quadex Automation Sdn Bhd</t>
+  </si>
+  <si>
+    <t>Jalan 16/11, 46350, Petaling Jaya, Selangor</t>
+  </si>
+  <si>
+    <t>P-250682-004M</t>
+  </si>
+  <si>
     <t>A18</t>
   </si>
   <si>
@@ -246,54 +470,6 @@
   </si>
   <si>
     <t>H24</t>
-  </si>
-  <si>
-    <t>YOUR COMPANY NAME</t>
-  </si>
-  <si>
-    <t>YOUR COMPANY</t>
-  </si>
-  <si>
-    <t>As per YOUR COMPANY General Purchase Terms and Conditions</t>
-  </si>
-  <si>
-    <t>YOUR COMPANY ADDRESS LINE 1</t>
-  </si>
-  <si>
-    <t>YOUR COMPANY ADDRESS LINE 2</t>
-  </si>
-  <si>
-    <t>YOUR COMPANY LOGO</t>
-  </si>
-  <si>
-    <t>E8 (PO no.)</t>
-  </si>
-  <si>
-    <t>Tel No.  : YOUR COMPANY TEL NO.</t>
-  </si>
-  <si>
-    <t>Fax No. : YOUR COMPANY FAX NO.</t>
-  </si>
-  <si>
-    <t>MANAGER</t>
-  </si>
-  <si>
-    <t>NOTE 1</t>
-  </si>
-  <si>
-    <t>NOTE 2</t>
-  </si>
-  <si>
-    <t>NOTE 3</t>
-  </si>
-  <si>
-    <t>REMARK 1</t>
-  </si>
-  <si>
-    <t>REMARK 2</t>
-  </si>
-  <si>
-    <t>REMARK 3</t>
   </si>
 </sst>
 </file>
@@ -1122,7 +1298,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="224">
+  <cellXfs count="223">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1639,9 +1815,6 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="9" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -1735,6 +1908,85 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9224" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF7837E6-1A1D-3960-4430-6486F472183B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="371475" y="152400"/>
+          <a:ext cx="2333625" cy="1047750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2108,34 +2360,32 @@
       <c r="C1" s="52"/>
       <c r="D1" s="52"/>
       <c r="G1" s="53" t="s">
-        <v>64</v>
+        <v>104</v>
       </c>
       <c r="H1" s="53"/>
       <c r="I1" s="53"/>
     </row>
-    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="54"/>
       <c r="B2" s="52"/>
       <c r="C2" s="52"/>
       <c r="D2" s="52"/>
-      <c r="G2" s="223" t="s">
-        <v>66</v>
-      </c>
-      <c r="H2" s="223"/>
-      <c r="I2" s="223"/>
+      <c r="G2" s="157" t="s">
+        <v>94</v>
+      </c>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
     </row>
     <row r="3" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="222" t="s">
-        <v>68</v>
-      </c>
+      <c r="A3" s="222"/>
       <c r="B3" s="222"/>
       <c r="C3" s="222"/>
       <c r="D3" s="222"/>
-      <c r="G3" s="223" t="s">
-        <v>67</v>
-      </c>
-      <c r="H3" s="223"/>
-      <c r="I3" s="223"/>
+      <c r="G3" s="157" t="s">
+        <v>105</v>
+      </c>
+      <c r="H3" s="157"/>
+      <c r="I3" s="157"/>
     </row>
     <row r="4" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="222"/>
@@ -2152,7 +2402,7 @@
       <c r="C5" s="51"/>
       <c r="D5" s="51"/>
       <c r="G5" s="157" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="H5" s="157"/>
       <c r="I5" s="157"/>
@@ -2163,7 +2413,7 @@
       <c r="C6" s="51"/>
       <c r="D6" s="51"/>
       <c r="G6" s="157" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="H6" s="157"/>
       <c r="I6" s="157"/>
@@ -2175,23 +2425,23 @@
     </row>
     <row r="8" spans="1:10" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="143" t="s">
-        <v>61</v>
+        <v>128</v>
       </c>
       <c r="B8" s="142"/>
       <c r="C8" s="142"/>
       <c r="D8" s="142"/>
       <c r="E8" s="156" t="s">
-        <v>69</v>
+        <v>106</v>
       </c>
       <c r="F8" s="142"/>
       <c r="G8" s="27" t="s">
         <v>8</v>
       </c>
       <c r="H8" s="120" t="s">
-        <v>50</v>
+        <v>117</v>
       </c>
       <c r="I8" s="28" t="s">
-        <v>39</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2199,24 +2449,24 @@
         <v>0</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="30"/>
       <c r="F9" s="30"/>
       <c r="G9" s="97" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="H9" s="155" t="s">
-        <v>48</v>
+        <v>115</v>
       </c>
       <c r="I9" s="98"/>
     </row>
     <row r="10" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="33"/>
       <c r="B10" s="5" t="s">
-        <v>56</v>
+        <v>123</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -2224,14 +2474,14 @@
       <c r="F10" s="5"/>
       <c r="G10" s="153"/>
       <c r="H10" s="147" t="s">
-        <v>49</v>
+        <v>116</v>
       </c>
       <c r="I10" s="154"/>
     </row>
     <row r="11" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="33"/>
       <c r="B11" s="5" t="s">
-        <v>57</v>
+        <v>124</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -2246,12 +2496,12 @@
     <row r="12" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="84"/>
       <c r="B12" s="5" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="5"/>
       <c r="G12" s="26" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="H12" s="163">
         <f>I51</f>
@@ -2262,75 +2512,75 @@
     </row>
     <row r="13" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="90" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="B13" s="82"/>
       <c r="C13" s="8" t="s">
-        <v>51</v>
+        <v>118</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="5"/>
       <c r="F13" s="118"/>
       <c r="G13" s="185" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="H13" s="185"/>
       <c r="I13" s="186"/>
     </row>
     <row r="14" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="90" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="128" t="s">
-        <v>52</v>
+        <v>119</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="5"/>
       <c r="F14" s="118"/>
       <c r="G14" s="116" t="s">
-        <v>64</v>
+        <v>104</v>
       </c>
       <c r="H14" s="116"/>
       <c r="I14" s="117"/>
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="128" t="s">
-        <v>53</v>
+        <v>120</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="118"/>
       <c r="G15" s="165" t="s">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="H15" s="165"/>
       <c r="I15" s="166"/>
     </row>
     <row r="16" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="50" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="91" t="s">
-        <v>54</v>
+        <v>121</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="118"/>
       <c r="G16" s="165" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="H16" s="165"/>
       <c r="I16" s="166"/>
     </row>
     <row r="17" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -2343,7 +2593,7 @@
     </row>
     <row r="18" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="141" t="s">
-        <v>40</v>
+        <v>107</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -2351,14 +2601,14 @@
       <c r="E18" s="8"/>
       <c r="F18" s="119"/>
       <c r="G18" s="151" t="s">
-        <v>46</v>
+        <v>113</v>
       </c>
       <c r="H18" s="151"/>
       <c r="I18" s="152"/>
     </row>
     <row r="19" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="83" t="s">
-        <v>65</v>
+        <v>97</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -2371,7 +2621,7 @@
     </row>
     <row r="20" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -2387,7 +2637,7 @@
     </row>
     <row r="21" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="132" t="s">
-        <v>41</v>
+        <v>108</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -2400,7 +2650,7 @@
     </row>
     <row r="22" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="83" t="s">
-        <v>65</v>
+        <v>97</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -2413,7 +2663,7 @@
     </row>
     <row r="23" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -2428,25 +2678,25 @@
     </row>
     <row r="24" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="33" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5" t="s">
-        <v>63</v>
+        <v>104</v>
       </c>
       <c r="D24" s="20"/>
       <c r="E24" s="20"/>
       <c r="F24" s="36"/>
       <c r="G24" s="144"/>
       <c r="H24" s="146" t="s">
-        <v>62</v>
+        <v>129</v>
       </c>
       <c r="I24" s="145"/>
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="33" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="5" t="str">
@@ -2478,10 +2728,10 @@
       <c r="F26" s="180"/>
       <c r="G26" s="181"/>
       <c r="H26" s="60" t="s">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="I26" s="61" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:10" s="62" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2519,7 +2769,7 @@
       <c r="B29" s="134"/>
       <c r="C29" s="135"/>
       <c r="D29" s="140" t="s">
-        <v>47</v>
+        <v>114</v>
       </c>
       <c r="E29" s="137"/>
       <c r="F29" s="137"/>
@@ -2542,22 +2792,22 @@
     </row>
     <row r="31" spans="1:10" s="15" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="107" t="s">
-        <v>42</v>
+        <v>109</v>
       </c>
       <c r="B31" s="101" t="s">
-        <v>43</v>
+        <v>110</v>
       </c>
       <c r="C31" s="65" t="s">
-        <v>44</v>
+        <v>111</v>
       </c>
       <c r="D31" s="129" t="s">
-        <v>58</v>
+        <v>125</v>
       </c>
       <c r="H31" s="127" t="s">
-        <v>45</v>
+        <v>112</v>
       </c>
       <c r="I31" s="126" t="s">
-        <v>59</v>
+        <v>126</v>
       </c>
       <c r="J31" s="16"/>
     </row>
@@ -2741,7 +2991,7 @@
       <c r="B51" s="110"/>
       <c r="C51" s="102"/>
       <c r="D51" s="92" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E51" s="93"/>
       <c r="F51" s="93"/>
@@ -2757,7 +3007,7 @@
       <c r="B52" s="101"/>
       <c r="C52" s="102"/>
       <c r="D52" s="94" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="E52" s="93"/>
       <c r="F52" s="93"/>
@@ -2770,10 +3020,10 @@
       <c r="B53" s="101"/>
       <c r="C53" s="102"/>
       <c r="D53" s="95" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="E53" s="96" t="s">
-        <v>60</v>
+        <v>127</v>
       </c>
       <c r="F53" s="93"/>
       <c r="G53" s="93"/>
@@ -2804,7 +3054,7 @@
     </row>
     <row r="56" spans="1:11" s="15" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="40" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="B56" s="41"/>
       <c r="C56" s="41"/>
@@ -2817,12 +3067,12 @@
     </row>
     <row r="57" spans="1:11" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="40" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="B57" s="41"/>
       <c r="C57" s="41"/>
       <c r="D57" s="41" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E57" s="41"/>
       <c r="F57" s="41"/>
@@ -2854,20 +3104,20 @@
       </c>
       <c r="G59" s="198"/>
       <c r="H59" s="173" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I59" s="174"/>
     </row>
     <row r="60" spans="1:11" s="15" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="168" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B60" s="169"/>
       <c r="C60" s="169"/>
       <c r="D60" s="170"/>
       <c r="E60" s="169"/>
       <c r="F60" s="43" t="s">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="G60" s="44"/>
       <c r="H60" s="175"/>
@@ -2875,14 +3125,14 @@
     </row>
     <row r="61" spans="1:11" s="15" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="168" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B61" s="169"/>
       <c r="C61" s="169"/>
       <c r="D61" s="170"/>
       <c r="E61" s="169"/>
       <c r="F61" s="171" t="s">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="G61" s="161"/>
       <c r="H61" s="45"/>
@@ -2890,7 +3140,7 @@
     </row>
     <row r="62" spans="1:11" s="15" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="158" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B62" s="159"/>
       <c r="C62" s="160"/>
@@ -2903,14 +3153,14 @@
     </row>
     <row r="63" spans="1:11" s="15" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="204" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B63" s="205"/>
       <c r="C63" s="205"/>
       <c r="D63" s="213"/>
       <c r="E63" s="205"/>
       <c r="F63" s="49" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="G63" s="121" t="str">
         <f>H8</f>
@@ -2952,19 +3202,19 @@
       <c r="E66" s="209"/>
       <c r="F66" s="209"/>
       <c r="G66" s="74" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H66" s="122" t="str">
         <f>H8</f>
         <v>H8 (date)</v>
       </c>
       <c r="I66" s="28" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="210" t="s">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="B67" s="211"/>
       <c r="C67" s="211"/>
@@ -2974,7 +3224,7 @@
       <c r="G67" s="211"/>
       <c r="H67" s="212"/>
       <c r="I67" s="66" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2982,7 +3232,7 @@
         <v>1</v>
       </c>
       <c r="B68" s="187" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C68" s="188"/>
       <c r="D68" s="188"/>
@@ -2991,12 +3241,14 @@
       <c r="G68" s="188"/>
       <c r="H68" s="189"/>
       <c r="I68" s="19" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="17"/>
-      <c r="B69" s="199"/>
+      <c r="B69" s="199" t="s">
+        <v>99</v>
+      </c>
       <c r="C69" s="200"/>
       <c r="D69" s="200"/>
       <c r="E69" s="200"/>
@@ -3007,10 +3259,15 @@
     </row>
     <row r="70" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="67"/>
-      <c r="B70" s="11"/>
+      <c r="B70" s="11" t="s">
+        <v>83</v>
+      </c>
       <c r="C70" s="14"/>
       <c r="D70" s="14"/>
-      <c r="E70" s="68"/>
+      <c r="E70" s="68" t="str">
+        <f>E8</f>
+        <v>P-250682-004M</v>
+      </c>
       <c r="F70" s="13"/>
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
@@ -3032,7 +3289,7 @@
         <v>2</v>
       </c>
       <c r="B72" s="187" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="C72" s="188"/>
       <c r="D72" s="188"/>
@@ -3041,12 +3298,14 @@
       <c r="G72" s="188"/>
       <c r="H72" s="189"/>
       <c r="I72" s="19" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="67"/>
-      <c r="B73" s="199"/>
+      <c r="B73" s="199" t="s">
+        <v>100</v>
+      </c>
       <c r="C73" s="200"/>
       <c r="D73" s="200"/>
       <c r="E73" s="200"/>
@@ -3057,10 +3316,15 @@
     </row>
     <row r="74" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="17"/>
-      <c r="B74" s="11"/>
+      <c r="B74" s="11" t="s">
+        <v>83</v>
+      </c>
       <c r="C74" s="14"/>
       <c r="D74" s="14"/>
-      <c r="E74" s="69"/>
+      <c r="E74" s="69" t="str">
+        <f>E8</f>
+        <v>P-250682-004M</v>
+      </c>
       <c r="F74" s="13"/>
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
@@ -3082,7 +3346,7 @@
         <v>3</v>
       </c>
       <c r="B76" s="187" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C76" s="188"/>
       <c r="D76" s="188"/>
@@ -3091,7 +3355,7 @@
       <c r="G76" s="188"/>
       <c r="H76" s="189"/>
       <c r="I76" s="19" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3106,19 +3370,27 @@
       <c r="I77" s="19"/>
     </row>
     <row r="78" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="18"/>
-      <c r="B78" s="187"/>
+      <c r="A78" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B78" s="187" t="s">
+        <v>47</v>
+      </c>
       <c r="C78" s="188"/>
       <c r="D78" s="188"/>
       <c r="E78" s="188"/>
       <c r="F78" s="188"/>
       <c r="G78" s="188"/>
       <c r="H78" s="189"/>
-      <c r="I78" s="19"/>
+      <c r="I78" s="19" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="79" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="17"/>
-      <c r="B79" s="187"/>
+      <c r="B79" s="187" t="s">
+        <v>28</v>
+      </c>
       <c r="C79" s="188"/>
       <c r="D79" s="188"/>
       <c r="E79" s="188"/>
@@ -3139,15 +3411,21 @@
       <c r="I80" s="19"/>
     </row>
     <row r="81" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="18"/>
-      <c r="B81" s="187"/>
+      <c r="A81" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B81" s="187" t="s">
+        <v>26</v>
+      </c>
       <c r="C81" s="188"/>
       <c r="D81" s="188"/>
       <c r="E81" s="188"/>
       <c r="F81" s="188"/>
       <c r="G81" s="188"/>
       <c r="H81" s="189"/>
-      <c r="I81" s="19"/>
+      <c r="I81" s="19" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="82" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="17"/>
@@ -3161,19 +3439,27 @@
       <c r="I82" s="19"/>
     </row>
     <row r="83" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="18"/>
-      <c r="B83" s="187"/>
+      <c r="A83" s="18">
+        <v>4</v>
+      </c>
+      <c r="B83" s="187" t="s">
+        <v>54</v>
+      </c>
       <c r="C83" s="188"/>
       <c r="D83" s="188"/>
       <c r="E83" s="188"/>
       <c r="F83" s="188"/>
       <c r="G83" s="188"/>
       <c r="H83" s="189"/>
-      <c r="I83" s="19"/>
+      <c r="I83" s="19" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="84" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="17"/>
-      <c r="B84" s="187"/>
+      <c r="B84" s="187" t="s">
+        <v>55</v>
+      </c>
       <c r="C84" s="188"/>
       <c r="D84" s="188"/>
       <c r="E84" s="188"/>
@@ -3194,19 +3480,27 @@
       <c r="I85" s="19"/>
     </row>
     <row r="86" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="18"/>
-      <c r="B86" s="187"/>
+      <c r="A86" s="18">
+        <v>5</v>
+      </c>
+      <c r="B86" s="187" t="s">
+        <v>27</v>
+      </c>
       <c r="C86" s="188"/>
       <c r="D86" s="188"/>
       <c r="E86" s="188"/>
       <c r="F86" s="188"/>
       <c r="G86" s="188"/>
       <c r="H86" s="189"/>
-      <c r="I86" s="19"/>
+      <c r="I86" s="19" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="87" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="18"/>
-      <c r="B87" s="187"/>
+      <c r="B87" s="187" t="s">
+        <v>56</v>
+      </c>
       <c r="C87" s="188"/>
       <c r="D87" s="188"/>
       <c r="E87" s="188"/>
@@ -3217,7 +3511,9 @@
     </row>
     <row r="88" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="18"/>
-      <c r="B88" s="187"/>
+      <c r="B88" s="187" t="s">
+        <v>57</v>
+      </c>
       <c r="C88" s="188"/>
       <c r="D88" s="188"/>
       <c r="E88" s="188"/>
@@ -3238,19 +3534,27 @@
       <c r="I89" s="19"/>
     </row>
     <row r="90" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="18"/>
-      <c r="B90" s="187"/>
+      <c r="A90" s="18">
+        <v>6</v>
+      </c>
+      <c r="B90" s="187" t="s">
+        <v>59</v>
+      </c>
       <c r="C90" s="188"/>
       <c r="D90" s="188"/>
       <c r="E90" s="188"/>
       <c r="F90" s="188"/>
       <c r="G90" s="188"/>
       <c r="H90" s="189"/>
-      <c r="I90" s="19"/>
+      <c r="I90" s="19" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="91" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="17"/>
-      <c r="B91" s="187"/>
+      <c r="B91" s="187" t="s">
+        <v>60</v>
+      </c>
       <c r="C91" s="188"/>
       <c r="D91" s="188"/>
       <c r="E91" s="188"/>
@@ -3271,15 +3575,21 @@
       <c r="I92" s="19"/>
     </row>
     <row r="93" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="18"/>
-      <c r="B93" s="187"/>
+      <c r="A93" s="18">
+        <v>7</v>
+      </c>
+      <c r="B93" s="187" t="s">
+        <v>31</v>
+      </c>
       <c r="C93" s="188"/>
       <c r="D93" s="188"/>
       <c r="E93" s="188"/>
       <c r="F93" s="188"/>
       <c r="G93" s="188"/>
       <c r="H93" s="189"/>
-      <c r="I93" s="19"/>
+      <c r="I93" s="19" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="94" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="17"/>
@@ -3293,8 +3603,12 @@
       <c r="I94" s="19"/>
     </row>
     <row r="95" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="18"/>
-      <c r="B95" s="187"/>
+      <c r="A95" s="18">
+        <v>8</v>
+      </c>
+      <c r="B95" s="187" t="s">
+        <v>32</v>
+      </c>
       <c r="C95" s="188"/>
       <c r="D95" s="188"/>
       <c r="E95" s="188"/>
@@ -3304,59 +3618,113 @@
       <c r="I95" s="19"/>
     </row>
     <row r="96" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="18"/>
-      <c r="B96" s="187"/>
+      <c r="A96" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B96" s="187" t="s">
+        <v>44</v>
+      </c>
       <c r="C96" s="188"/>
       <c r="D96" s="188"/>
       <c r="E96" s="188"/>
       <c r="F96" s="188"/>
       <c r="G96" s="188"/>
       <c r="H96" s="189"/>
-      <c r="I96" s="19"/>
+      <c r="I96" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="97" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="18"/>
-      <c r="B97" s="187"/>
-      <c r="C97" s="188"/>
-      <c r="D97" s="188"/>
-      <c r="E97" s="188"/>
-      <c r="F97" s="188"/>
-      <c r="G97" s="188"/>
-      <c r="H97" s="189"/>
-      <c r="I97" s="19"/>
+      <c r="A97" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B97" s="187" t="s">
+        <v>52</v>
+      </c>
+      <c r="C97" s="188" t="s">
+        <v>16</v>
+      </c>
+      <c r="D97" s="188" t="s">
+        <v>16</v>
+      </c>
+      <c r="E97" s="188" t="s">
+        <v>16</v>
+      </c>
+      <c r="F97" s="188" t="s">
+        <v>16</v>
+      </c>
+      <c r="G97" s="188" t="s">
+        <v>16</v>
+      </c>
+      <c r="H97" s="189" t="s">
+        <v>16</v>
+      </c>
+      <c r="I97" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="98" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="18"/>
-      <c r="B98" s="11"/>
+      <c r="A98" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B98" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="C98" s="14"/>
       <c r="D98" s="14"/>
       <c r="E98" s="14"/>
       <c r="F98" s="14"/>
       <c r="G98" s="14"/>
       <c r="H98" s="32"/>
-      <c r="I98" s="19"/>
+      <c r="I98" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="99" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="18"/>
-      <c r="B99" s="11"/>
+      <c r="A99" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B99" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C99" s="14"/>
       <c r="D99" s="14"/>
       <c r="E99" s="14"/>
       <c r="F99" s="14"/>
       <c r="G99" s="14"/>
       <c r="H99" s="32"/>
-      <c r="I99" s="19"/>
+      <c r="I99" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="100" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="18"/>
-      <c r="B100" s="187"/>
-      <c r="C100" s="188"/>
-      <c r="D100" s="188"/>
-      <c r="E100" s="188"/>
-      <c r="F100" s="188"/>
-      <c r="G100" s="188"/>
-      <c r="H100" s="189"/>
-      <c r="I100" s="19"/>
+      <c r="A100" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B100" s="187" t="s">
+        <v>101</v>
+      </c>
+      <c r="C100" s="188" t="s">
+        <v>19</v>
+      </c>
+      <c r="D100" s="188" t="s">
+        <v>19</v>
+      </c>
+      <c r="E100" s="188" t="s">
+        <v>19</v>
+      </c>
+      <c r="F100" s="188" t="s">
+        <v>19</v>
+      </c>
+      <c r="G100" s="188" t="s">
+        <v>19</v>
+      </c>
+      <c r="H100" s="189" t="s">
+        <v>19</v>
+      </c>
+      <c r="I100" s="19" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="101" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="18"/>
@@ -3370,8 +3738,12 @@
       <c r="I101" s="19"/>
     </row>
     <row r="102" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="18"/>
-      <c r="B102" s="187"/>
+      <c r="A102" s="18">
+        <v>9</v>
+      </c>
+      <c r="B102" s="187" t="s">
+        <v>37</v>
+      </c>
       <c r="C102" s="188"/>
       <c r="D102" s="188"/>
       <c r="E102" s="188"/>
@@ -3392,19 +3764,27 @@
       <c r="I103" s="21"/>
     </row>
     <row r="104" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="18"/>
-      <c r="B104" s="11"/>
+      <c r="A104" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B104" s="11" t="s">
+        <v>69</v>
+      </c>
       <c r="C104" s="20"/>
       <c r="D104" s="20"/>
       <c r="E104" s="20"/>
       <c r="F104" s="194"/>
       <c r="G104" s="194"/>
       <c r="H104" s="195"/>
-      <c r="I104" s="19"/>
+      <c r="I104" s="19" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="105" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="18"/>
-      <c r="B105" s="12"/>
+      <c r="B105" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="C105" s="13"/>
       <c r="D105" s="70"/>
       <c r="E105" s="70"/>
@@ -3425,8 +3805,12 @@
       <c r="I106" s="21"/>
     </row>
     <row r="107" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="18"/>
-      <c r="B107" s="187"/>
+      <c r="A107" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B107" s="187" t="s">
+        <v>49</v>
+      </c>
       <c r="C107" s="188"/>
       <c r="D107" s="188"/>
       <c r="E107" s="188"/>
@@ -3437,18 +3821,24 @@
     </row>
     <row r="108" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="18"/>
-      <c r="B108" s="187"/>
+      <c r="B108" s="187" t="s">
+        <v>50</v>
+      </c>
       <c r="C108" s="188"/>
       <c r="D108" s="188"/>
       <c r="E108" s="188"/>
       <c r="F108" s="188"/>
       <c r="G108" s="188"/>
       <c r="H108" s="189"/>
-      <c r="I108" s="19"/>
+      <c r="I108" s="19" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="109" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="18"/>
-      <c r="B109" s="193"/>
+      <c r="B109" s="193" t="s">
+        <v>66</v>
+      </c>
       <c r="C109" s="188"/>
       <c r="D109" s="188"/>
       <c r="E109" s="188"/>
@@ -3457,12 +3847,18 @@
       <c r="H109" s="189"/>
       <c r="I109" s="19"/>
     </row>
-    <row r="110" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="18"/>
-      <c r="B110" s="187"/>
+      <c r="B110" s="187" t="s">
+        <v>53</v>
+      </c>
       <c r="C110" s="188"/>
-      <c r="D110" s="188"/>
-      <c r="E110" s="188"/>
+      <c r="D110" s="188" t="s">
+        <v>10</v>
+      </c>
+      <c r="E110" s="188" t="s">
+        <v>11</v>
+      </c>
       <c r="F110" s="188"/>
       <c r="G110" s="188"/>
       <c r="H110" s="189"/>
@@ -3480,19 +3876,29 @@
       <c r="I111" s="19"/>
     </row>
     <row r="112" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="18"/>
-      <c r="B112" s="187"/>
+      <c r="A112" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B112" s="187" t="s">
+        <v>14</v>
+      </c>
       <c r="C112" s="188"/>
       <c r="D112" s="188"/>
-      <c r="E112" s="188"/>
+      <c r="E112" s="188" t="s">
+        <v>15</v>
+      </c>
       <c r="F112" s="188"/>
       <c r="G112" s="188"/>
       <c r="H112" s="189"/>
-      <c r="I112" s="19"/>
+      <c r="I112" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="113" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="18"/>
-      <c r="B113" s="190"/>
+      <c r="B113" s="190" t="s">
+        <v>64</v>
+      </c>
       <c r="C113" s="191"/>
       <c r="D113" s="191"/>
       <c r="E113" s="191"/>
@@ -3506,10 +3912,10 @@
       <c r="B114" s="187"/>
       <c r="C114" s="188"/>
       <c r="D114" s="188" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E114" s="188" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F114" s="188"/>
       <c r="G114" s="188"/>
@@ -3517,22 +3923,34 @@
       <c r="I114" s="19"/>
     </row>
     <row r="115" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="18"/>
-      <c r="B115" s="187"/>
+      <c r="A115" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B115" s="187" t="s">
+        <v>62</v>
+      </c>
       <c r="C115" s="188"/>
       <c r="D115" s="188"/>
-      <c r="E115" s="188"/>
+      <c r="E115" s="188" t="s">
+        <v>20</v>
+      </c>
       <c r="F115" s="188"/>
       <c r="G115" s="188"/>
       <c r="H115" s="189"/>
-      <c r="I115" s="19"/>
+      <c r="I115" s="19" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="116" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="18"/>
-      <c r="B116" s="187"/>
+      <c r="B116" s="187" t="s">
+        <v>63</v>
+      </c>
       <c r="C116" s="188"/>
       <c r="D116" s="188"/>
-      <c r="E116" s="188"/>
+      <c r="E116" s="188" t="s">
+        <v>21</v>
+      </c>
       <c r="F116" s="188"/>
       <c r="G116" s="188"/>
       <c r="H116" s="189"/>
@@ -3540,7 +3958,9 @@
     </row>
     <row r="117" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="18"/>
-      <c r="B117" s="187"/>
+      <c r="B117" s="187" t="s">
+        <v>65</v>
+      </c>
       <c r="C117" s="188"/>
       <c r="D117" s="188"/>
       <c r="E117" s="188"/>
@@ -3561,19 +3981,27 @@
       <c r="I118" s="19"/>
     </row>
     <row r="119" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="18"/>
-      <c r="B119" s="187"/>
+      <c r="A119" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B119" s="187" t="s">
+        <v>74</v>
+      </c>
       <c r="C119" s="188"/>
       <c r="D119" s="188"/>
       <c r="E119" s="188"/>
       <c r="F119" s="188"/>
       <c r="G119" s="188"/>
       <c r="H119" s="189"/>
-      <c r="I119" s="19"/>
+      <c r="I119" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="120" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="18"/>
-      <c r="B120" s="187"/>
+      <c r="B120" s="187" t="s">
+        <v>61</v>
+      </c>
       <c r="C120" s="188"/>
       <c r="D120" s="188"/>
       <c r="E120" s="188"/>
@@ -3710,5 +4138,6 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="65" max="8" man="1"/>
   </rowBreaks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>